<commit_message>
feat: enhance selection workflow and developer library
</commit_message>
<xml_diff>
--- a/analysis/开发人维度/于林_sku_report.xlsx
+++ b/analysis/开发人维度/于林_sku_report.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S2"/>
+  <dimension ref="A1:T2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -445,70 +445,75 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
+          <t>总结算销售额</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
           <t>总利润率</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>总可用库存</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>存活率</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>存活sku销售量</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>存活sku销售额</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>存活SKU数</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>留存SKU总利润</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>留存SKU利润率</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>淘汰SKU销售量</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>淘汰SKU销售额</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>淘汰SKU总数</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>淘汰率</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>淘汰SKU总利润</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>淘汰SKU利润率</t>
         </is>
@@ -524,46 +529,46 @@
         <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>113</v>
+        <v>177</v>
       </c>
       <c r="D2" t="n">
-        <v>1442.45</v>
+        <v>2255.41</v>
       </c>
       <c r="E2" t="n">
-        <v>94.77</v>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>6.57%</t>
-        </is>
-      </c>
-      <c r="G2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H2" t="inlineStr">
+        <v>165.28</v>
+      </c>
+      <c r="F2" t="n">
+        <v>1888.84</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>8.75%</t>
+        </is>
+      </c>
+      <c r="H2" t="n">
+        <v>11</v>
+      </c>
+      <c r="I2" t="inlineStr">
         <is>
           <t>100.00%</t>
         </is>
       </c>
-      <c r="I2" t="n">
-        <v>113</v>
-      </c>
       <c r="J2" t="n">
-        <v>1442.45</v>
+        <v>177</v>
       </c>
       <c r="K2" t="n">
+        <v>2255.41</v>
+      </c>
+      <c r="L2" t="n">
         <v>1</v>
       </c>
-      <c r="L2" t="n">
-        <v>94.77</v>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>6.57%</t>
-        </is>
-      </c>
-      <c r="N2" t="n">
-        <v>0</v>
+      <c r="M2" t="n">
+        <v>165.28</v>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>8.75%</t>
+        </is>
       </c>
       <c r="O2" t="n">
         <v>0</v>
@@ -571,15 +576,18 @@
       <c r="P2" t="n">
         <v>0</v>
       </c>
-      <c r="Q2" t="inlineStr">
+      <c r="Q2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R2" t="inlineStr">
         <is>
           <t>0.00%</t>
         </is>
       </c>
-      <c r="R2" t="n">
+      <c r="S2" t="n">
         <v>0</v>
       </c>
-      <c r="S2" t="inlineStr">
+      <c r="T2" t="inlineStr">
         <is>
           <t>0.00%</t>
         </is>
@@ -596,7 +604,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:I2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -632,10 +640,15 @@
       </c>
       <c r="G1" t="inlineStr">
         <is>
+          <t>总结算销售额</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
           <t>总可用库存</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>最新标签</t>
         </is>
@@ -658,18 +671,21 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>113</v>
+        <v>177</v>
       </c>
       <c r="E2" t="n">
-        <v>1442.45</v>
+        <v>2255.41</v>
       </c>
       <c r="F2" t="n">
-        <v>94.77</v>
+        <v>165.28</v>
       </c>
       <c r="G2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H2" t="inlineStr">
+        <v>1888.84417616812</v>
+      </c>
+      <c r="H2" t="n">
+        <v>11</v>
+      </c>
+      <c r="I2" t="inlineStr">
         <is>
           <t>欧洲精铺2025</t>
         </is>

</xml_diff>